<commit_message>
Extends the "example" dataset with more meaningful entries, and also defines reserves and a monthly income.
</commit_message>
<xml_diff>
--- a/data/example/output/dataset.analysis.xlsx
+++ b/data/example/output/dataset.analysis.xlsx
@@ -984,7 +984,7 @@
         </is>
       </c>
       <c r="F7" s="5" t="n">
-        <v>11166.35</v>
+        <v>18300</v>
       </c>
       <c r="G7" s="5" t="n">
         <v>1888.95</v>
@@ -1003,7 +1003,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>11166.35</v>
+        <v>18300</v>
       </c>
       <c r="C8" s="5" t="n">
         <v>0</v>
@@ -1020,7 +1020,7 @@
         <v>0</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>3104.36</v>
+        <v>9674.959999999999</v>
       </c>
       <c r="I8" s="5" t="n">
         <v>0</v>
@@ -1036,7 +1036,7 @@
         <v>0</v>
       </c>
       <c r="C9" s="5" t="n">
-        <v>3104.36</v>
+        <v>9674.959999999999</v>
       </c>
     </row>
     <row r="10">
@@ -1059,10 +1059,10 @@
         </is>
       </c>
       <c r="B11" s="7" t="n">
-        <v>13055.3</v>
+        <v>20188.95</v>
       </c>
       <c r="C11" s="7" t="n">
-        <v>3104.36</v>
+        <v>9674.959999999999</v>
       </c>
     </row>
     <row r="13">
@@ -1085,10 +1085,10 @@
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>13505.3</v>
+        <v>20638.95</v>
       </c>
       <c r="C15" s="7" t="n">
-        <v>3104.36</v>
+        <v>9674.959999999999</v>
       </c>
     </row>
   </sheetData>
@@ -1150,7 +1150,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>11166.35</v>
+        <v>18300</v>
       </c>
     </row>
     <row r="27">
@@ -1179,57 +1179,57 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>1893.02</v>
+        <v>7215.02</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Leben</t>
+          <t>Einkaufen</t>
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>452.55</v>
+        <v>1556.79</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Einkaufen</t>
+          <t>Leben</t>
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>371.69</v>
+        <v>437.55</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Freizeit</t>
+          <t>Finanzen</t>
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>153.5</v>
+        <v>173.5</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Mobilität</t>
+          <t>Freizeit</t>
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>123.6</v>
+        <v>168.5</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Finanzen</t>
+          <t>Mobilität</t>
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>110</v>
+        <v>123.6</v>
       </c>
     </row>
     <row r="49">
@@ -1293,7 +1293,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D38"/>
+  <dimension ref="A1:D46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1348,344 +1348,472 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Mobilität</t>
+          <t>Einkommen</t>
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>0</v>
+        <v>4200</v>
       </c>
       <c r="C8" s="5" t="n">
-        <v>26.7</v>
+        <v>0</v>
       </c>
       <c r="D8" s="5" t="n">
-        <v>-26.7</v>
+        <v>4200</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Leben</t>
+          <t>Wohnen</t>
         </is>
       </c>
       <c r="B9" s="5" t="n">
         <v>0</v>
       </c>
       <c r="C9" s="5" t="n">
-        <v>19</v>
+        <v>1787.9</v>
       </c>
       <c r="D9" s="5" t="n">
-        <v>-19</v>
+        <v>-1787.9</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Wohnen</t>
+          <t>Einkaufen</t>
         </is>
       </c>
       <c r="B10" s="5" t="n">
         <v>0</v>
       </c>
       <c r="C10" s="5" t="n">
-        <v>13.9</v>
+        <v>388.75</v>
       </c>
       <c r="D10" s="5" t="n">
-        <v>-13.9</v>
+        <v>-388.75</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>Mobilität</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>-26.7</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Leben</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>-19</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>Rückerstattungen</t>
         </is>
       </c>
-      <c r="B11" s="5" t="n">
+      <c r="B13" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="C11" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" s="5" t="n">
+      <c r="C13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="5" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>February 2025</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>Credit in CHF</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>Debit in CHF</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>Net in CHF</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Einkommen</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>4200</v>
+      </c>
+      <c r="C19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="5" t="n">
+        <v>4200</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Wohnen</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="5" t="n">
+        <v>1774</v>
+      </c>
+      <c r="D20" s="5" t="n">
+        <v>-1774</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Einkaufen</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="5" t="n">
+        <v>434.7</v>
+      </c>
+      <c r="D21" s="5" t="n">
+        <v>-434.7</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
         <is>
           <t>Freizeit</t>
         </is>
       </c>
-      <c r="B17" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C17" s="5" t="n">
+      <c r="B22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="D17" s="5" t="n">
+      <c r="D22" s="5" t="n">
         <v>-3</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>March 2025</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B22" s="4" t="inlineStr">
+      <c r="B27" s="4" t="inlineStr">
         <is>
           <t>Credit in CHF</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr">
+      <c r="C27" s="4" t="inlineStr">
         <is>
           <t>Debit in CHF</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
+      <c r="D27" s="4" t="inlineStr">
         <is>
           <t>Net in CHF</t>
         </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Einkommen</t>
-        </is>
-      </c>
-      <c r="B23" s="5" t="n">
-        <v>6966.35</v>
-      </c>
-      <c r="C23" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D23" s="5" t="n">
-        <v>6966.35</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Leben</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="n">
-        <v>1787.95</v>
-      </c>
-      <c r="C24" s="5" t="n">
-        <v>433.55</v>
-      </c>
-      <c r="D24" s="5" t="n">
-        <v>1354.4</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Wohnen</t>
-        </is>
-      </c>
-      <c r="B25" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C25" s="5" t="n">
-        <v>1879.12</v>
-      </c>
-      <c r="D25" s="5" t="n">
-        <v>-1879.12</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Einkaufen</t>
-        </is>
-      </c>
-      <c r="B26" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C26" s="5" t="n">
-        <v>371.69</v>
-      </c>
-      <c r="D26" s="5" t="n">
-        <v>-371.69</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Freizeit</t>
-        </is>
-      </c>
-      <c r="B27" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C27" s="5" t="n">
-        <v>150.5</v>
-      </c>
-      <c r="D27" s="5" t="n">
-        <v>-150.5</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Mobilität</t>
+          <t>Einkommen</t>
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>0</v>
+        <v>5700</v>
       </c>
       <c r="C28" s="5" t="n">
-        <v>96.90000000000001</v>
+        <v>0</v>
       </c>
       <c r="D28" s="5" t="n">
-        <v>-96.90000000000001</v>
+        <v>5700</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Finanzen</t>
+          <t>Leben</t>
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>0</v>
+        <v>1787.95</v>
       </c>
       <c r="C29" s="5" t="n">
-        <v>85</v>
+        <v>418.55</v>
       </c>
       <c r="D29" s="5" t="n">
-        <v>-85</v>
+        <v>1369.4</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t>Wohnen</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="5" t="n">
+        <v>1879.12</v>
+      </c>
+      <c r="D30" s="5" t="n">
+        <v>-1879.12</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Einkaufen</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="5" t="n">
+        <v>371.69</v>
+      </c>
+      <c r="D31" s="5" t="n">
+        <v>-371.69</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Freizeit</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="5" t="n">
+        <v>165.5</v>
+      </c>
+      <c r="D32" s="5" t="n">
+        <v>-165.5</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Mobilität</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="5" t="n">
+        <v>96.90000000000001</v>
+      </c>
+      <c r="D33" s="5" t="n">
+        <v>-96.90000000000001</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
           <t>Uncategorized</t>
         </is>
       </c>
-      <c r="B30" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C30" s="5" t="n">
+      <c r="B34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="5" t="n">
         <v>12.4</v>
       </c>
-      <c r="D30" s="5" t="n">
+      <c r="D34" s="5" t="n">
         <v>-12.4</v>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="3" t="inlineStr">
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Finanzen</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="D35" s="5" t="n">
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
         <is>
           <t>April 2025</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="4" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B35" s="4" t="inlineStr">
+      <c r="B40" s="4" t="inlineStr">
         <is>
           <t>Credit in CHF</t>
         </is>
       </c>
-      <c r="C35" s="4" t="inlineStr">
+      <c r="C40" s="4" t="inlineStr">
         <is>
           <t>Debit in CHF</t>
         </is>
       </c>
-      <c r="D35" s="4" t="inlineStr">
+      <c r="D40" s="4" t="inlineStr">
         <is>
           <t>Net in CHF</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
+    <row r="41">
+      <c r="A41" t="inlineStr">
         <is>
           <t>Einkommen</t>
         </is>
       </c>
-      <c r="B36" s="5" t="n">
+      <c r="B41" s="5" t="n">
         <v>4200</v>
       </c>
-      <c r="C36" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D36" s="5" t="n">
+      <c r="C41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D41" s="5" t="n">
         <v>4200</v>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Wohnen</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="5" t="n">
+        <v>1774</v>
+      </c>
+      <c r="D42" s="5" t="n">
+        <v>-1774</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Einkaufen</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="5" t="n">
+        <v>361.65</v>
+      </c>
+      <c r="D43" s="5" t="n">
+        <v>-361.65</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Finanzen</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="5" t="n">
+        <v>168.5</v>
+      </c>
+      <c r="D44" s="5" t="n">
+        <v>-168.5</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Uncategorized</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>69.05</v>
+      </c>
+      <c r="C45" s="5" t="n">
+        <v>46.2</v>
+      </c>
+      <c r="D45" s="5" t="n">
+        <v>22.85</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
         <is>
           <t>Freizeit</t>
         </is>
       </c>
-      <c r="B37" s="5" t="n">
+      <c r="B46" s="5" t="n">
         <v>100</v>
       </c>
-      <c r="C37" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D37" s="5" t="n">
+      <c r="C46" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D46" s="5" t="n">
         <v>100</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>Finanzen</t>
-        </is>
-      </c>
-      <c r="B38" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C38" s="5" t="n">
-        <v>25</v>
-      </c>
-      <c r="D38" s="5" t="n">
-        <v>-25</v>
       </c>
     </row>
   </sheetData>
@@ -1699,7 +1827,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1760,586 +1888,775 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Leben</t>
+          <t>Einkaufen</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Familie</t>
+          <t>Supermärkte</t>
         </is>
       </c>
       <c r="C8" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D8" s="5" t="n">
-        <v>19</v>
+        <v>388.75</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>-19</v>
+        <v>-388.75</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Mobilität</t>
+          <t>Einkommen</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Privater Verkehr</t>
+          <t>Lohn</t>
         </is>
       </c>
       <c r="C9" s="5" t="n">
-        <v>0</v>
+        <v>4200</v>
       </c>
       <c r="D9" s="5" t="n">
-        <v>26.7</v>
+        <v>0</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>-26.7</v>
+        <v>4200</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>Leben</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Familie</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>-19</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Mobilität</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Privater Verkehr</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>-26.7</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>Wohnen</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Miete und Hypothek</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>1774</v>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>-1774</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Wohnen</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
         <is>
           <t>Haushalt</t>
         </is>
       </c>
-      <c r="C10" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" s="5" t="n">
+      <c r="C13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="5" t="n">
         <v>13.9</v>
       </c>
-      <c r="E10" s="5" t="n">
+      <c r="E13" s="5" t="n">
         <v>-13.9</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>February 2025</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>Subcategory</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>Credit in CHF</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>Debit in CHF</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>Net in CHF</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Einkaufen</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Supermärkte</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="5" t="n">
+        <v>434.7</v>
+      </c>
+      <c r="E19" s="5" t="n">
+        <v>-434.7</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Einkommen</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Lohn</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="n">
+        <v>4200</v>
+      </c>
+      <c r="D20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" s="5" t="n">
+        <v>4200</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
         <is>
           <t>Freizeit</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>Gastronomie</t>
         </is>
       </c>
-      <c r="C16" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D16" s="5" t="n">
+      <c r="C21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="E16" s="5" t="n">
+      <c r="E21" s="5" t="n">
         <v>-3</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>March 2025</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>Subcategory</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>Credit in CHF</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>Debit in CHF</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>Net in CHF</t>
-        </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Einkaufen</t>
+          <t>Wohnen</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Supermärkte</t>
+          <t>Miete und Hypothek</t>
         </is>
       </c>
       <c r="C22" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D22" s="5" t="n">
-        <v>189.75</v>
+        <v>1774</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>-189.75</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Einkaufen</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Detail-Lebensmittel</t>
-        </is>
-      </c>
-      <c r="C23" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D23" s="5" t="n">
-        <v>167.29</v>
-      </c>
-      <c r="E23" s="5" t="n">
-        <v>-167.29</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Einkaufen</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Sonstiges Einkaufen</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D24" s="5" t="n">
-        <v>14.65</v>
-      </c>
-      <c r="E24" s="5" t="n">
-        <v>-14.65</v>
+        <v>-1774</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Einkommen</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Lohn</t>
-        </is>
-      </c>
-      <c r="C25" s="5" t="n">
-        <v>6966.35</v>
-      </c>
-      <c r="D25" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E25" s="5" t="n">
-        <v>6966.35</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Finanzen</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Bargeldbezug</t>
-        </is>
-      </c>
-      <c r="C26" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D26" s="5" t="n">
-        <v>80</v>
-      </c>
-      <c r="E26" s="5" t="n">
-        <v>-80</v>
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>March 2025</t>
+        </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Finanzen</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Fees</t>
-        </is>
-      </c>
-      <c r="C27" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D27" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="E27" s="5" t="n">
-        <v>-5</v>
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>Subcategory</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>Credit in CHF</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>Debit in CHF</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>Net in CHF</t>
+        </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Freizeit</t>
+          <t>Einkaufen</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Gastronomie</t>
+          <t>Supermärkte</t>
         </is>
       </c>
       <c r="C28" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D28" s="5" t="n">
-        <v>150.5</v>
+        <v>189.75</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>-150.5</v>
+        <v>-189.75</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Leben</t>
+          <t>Einkaufen</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Gesundheit</t>
+          <t>Detail-Lebensmittel</t>
         </is>
       </c>
       <c r="C29" s="5" t="n">
-        <v>1787.95</v>
+        <v>0</v>
       </c>
       <c r="D29" s="5" t="n">
-        <v>101.85</v>
+        <v>167.29</v>
       </c>
       <c r="E29" s="5" t="n">
-        <v>1686.1</v>
+        <v>-167.29</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Leben</t>
+          <t>Einkaufen</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Familie</t>
+          <t>Sonstiges Einkaufen</t>
         </is>
       </c>
       <c r="C30" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D30" s="5" t="n">
-        <v>200</v>
+        <v>14.65</v>
       </c>
       <c r="E30" s="5" t="n">
-        <v>-200</v>
+        <v>-14.65</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Leben</t>
+          <t>Einkommen</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Styling und Wellness</t>
+          <t>Lohn</t>
         </is>
       </c>
       <c r="C31" s="5" t="n">
-        <v>0</v>
+        <v>5700</v>
       </c>
       <c r="D31" s="5" t="n">
-        <v>79.90000000000001</v>
+        <v>0</v>
       </c>
       <c r="E31" s="5" t="n">
-        <v>-79.90000000000001</v>
+        <v>5700</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Leben</t>
+          <t>Finanzen</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Sonstiges Leben</t>
+          <t>Fees</t>
         </is>
       </c>
       <c r="C32" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D32" s="5" t="n">
-        <v>51.8</v>
+        <v>5</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>-51.8</v>
+        <v>-5</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Mobilität</t>
+          <t>Freizeit</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Öffentlicher Verkehr</t>
+          <t>Gastronomie</t>
         </is>
       </c>
       <c r="C33" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D33" s="5" t="n">
-        <v>96.90000000000001</v>
+        <v>150.5</v>
       </c>
       <c r="E33" s="5" t="n">
-        <v>-96.90000000000001</v>
+        <v>-150.5</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Wohnen</t>
+          <t>Freizeit</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Miete und Hypothek</t>
+          <t>Kultur</t>
         </is>
       </c>
       <c r="C34" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D34" s="5" t="n">
-        <v>1774</v>
+        <v>15</v>
       </c>
       <c r="E34" s="5" t="n">
-        <v>-1774</v>
+        <v>-15</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Wohnen</t>
+          <t>Leben</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Kommunikation</t>
+          <t>Gesundheit</t>
         </is>
       </c>
       <c r="C35" s="5" t="n">
-        <v>0</v>
+        <v>1787.95</v>
       </c>
       <c r="D35" s="5" t="n">
-        <v>70.27</v>
+        <v>101.85</v>
       </c>
       <c r="E35" s="5" t="n">
-        <v>-70.27</v>
+        <v>1686.1</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Wohnen</t>
+          <t>Leben</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Haushalt</t>
+          <t>Familie</t>
         </is>
       </c>
       <c r="C36" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D36" s="5" t="n">
-        <v>23.95</v>
+        <v>200</v>
       </c>
       <c r="E36" s="5" t="n">
-        <v>-23.95</v>
+        <v>-200</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>Leben</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Styling und Wellness</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D37" s="5" t="n">
+        <v>79.90000000000001</v>
+      </c>
+      <c r="E37" s="5" t="n">
+        <v>-79.90000000000001</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Leben</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Sonstiges Leben</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D38" s="5" t="n">
+        <v>36.8</v>
+      </c>
+      <c r="E38" s="5" t="n">
+        <v>-36.8</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Mobilität</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Öffentlicher Verkehr</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D39" s="5" t="n">
+        <v>96.90000000000001</v>
+      </c>
+      <c r="E39" s="5" t="n">
+        <v>-96.90000000000001</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
           <t>Wohnen</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Handwerk und Garten</t>
-        </is>
-      </c>
-      <c r="C37" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D37" s="5" t="n">
-        <v>10.9</v>
-      </c>
-      <c r="E37" s="5" t="n">
-        <v>-10.9</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="3" t="inlineStr">
-        <is>
-          <t>April 2025</t>
-        </is>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Miete und Hypothek</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D40" s="5" t="n">
+        <v>1774</v>
+      </c>
+      <c r="E40" s="5" t="n">
+        <v>-1774</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Wohnen</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Kommunikation</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D41" s="5" t="n">
+        <v>70.27</v>
+      </c>
+      <c r="E41" s="5" t="n">
+        <v>-70.27</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="4" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="B42" s="4" t="inlineStr">
-        <is>
-          <t>Subcategory</t>
-        </is>
-      </c>
-      <c r="C42" s="4" t="inlineStr">
-        <is>
-          <t>Credit in CHF</t>
-        </is>
-      </c>
-      <c r="D42" s="4" t="inlineStr">
-        <is>
-          <t>Debit in CHF</t>
-        </is>
-      </c>
-      <c r="E42" s="4" t="inlineStr">
-        <is>
-          <t>Net in CHF</t>
-        </is>
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Wohnen</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Haushalt</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D42" s="5" t="n">
+        <v>23.95</v>
+      </c>
+      <c r="E42" s="5" t="n">
+        <v>-23.95</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
+          <t>Wohnen</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Handwerk und Garten</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D43" s="5" t="n">
+        <v>10.9</v>
+      </c>
+      <c r="E43" s="5" t="n">
+        <v>-10.9</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>April 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>Subcategory</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>Credit in CHF</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>Debit in CHF</t>
+        </is>
+      </c>
+      <c r="E48" s="4" t="inlineStr">
+        <is>
+          <t>Net in CHF</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Einkaufen</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Supermärkte</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D49" s="5" t="n">
+        <v>361.65</v>
+      </c>
+      <c r="E49" s="5" t="n">
+        <v>-361.65</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
           <t>Einkommen</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B50" t="inlineStr">
         <is>
           <t>Lohn</t>
         </is>
       </c>
-      <c r="C43" s="5" t="n">
+      <c r="C50" s="5" t="n">
         <v>4200</v>
       </c>
-      <c r="D43" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E43" s="5" t="n">
+      <c r="D50" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E50" s="5" t="n">
         <v>4200</v>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
+    <row r="51">
+      <c r="A51" t="inlineStr">
         <is>
           <t>Finanzen</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Bargeldbezug</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D51" s="5" t="n">
+        <v>143.5</v>
+      </c>
+      <c r="E51" s="5" t="n">
+        <v>-143.5</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Finanzen</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
         <is>
           <t>Spenden</t>
         </is>
       </c>
-      <c r="C44" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D44" s="5" t="n">
+      <c r="C52" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D52" s="5" t="n">
         <v>25</v>
       </c>
-      <c r="E44" s="5" t="n">
+      <c r="E52" s="5" t="n">
         <v>-25</v>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
+    <row r="53">
+      <c r="A53" t="inlineStr">
         <is>
           <t>Freizeit</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B53" t="inlineStr">
         <is>
           <t>Reisen und Erleben</t>
         </is>
       </c>
-      <c r="C45" s="5" t="n">
+      <c r="C53" s="5" t="n">
         <v>100</v>
       </c>
-      <c r="D45" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E45" s="5" t="n">
+      <c r="D53" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E53" s="5" t="n">
         <v>100</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Wohnen</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Miete und Hypothek</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D54" s="5" t="n">
+        <v>1774</v>
+      </c>
+      <c r="E54" s="5" t="n">
+        <v>-1774</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adds an "amounts" filter for rules, which must exactly match one or more amounts in transactions.
</commit_message>
<xml_diff>
--- a/data/example/output/dataset.analysis.xlsx
+++ b/data/example/output/dataset.analysis.xlsx
@@ -987,7 +987,7 @@
         <v>18300</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>1888.95</v>
+        <v>2023.95</v>
       </c>
       <c r="H7" s="5" t="n">
         <v>0</v>
@@ -1046,7 +1046,7 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>1888.95</v>
+        <v>2023.95</v>
       </c>
       <c r="C10" s="5" t="n">
         <v>0</v>
@@ -1059,7 +1059,7 @@
         </is>
       </c>
       <c r="B11" s="7" t="n">
-        <v>20188.95</v>
+        <v>20323.95</v>
       </c>
       <c r="C11" s="7" t="n">
         <v>9674.959999999999</v>
@@ -1085,7 +1085,7 @@
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>20638.95</v>
+        <v>20773.95</v>
       </c>
       <c r="C15" s="7" t="n">
         <v>9674.959999999999</v>
@@ -1258,7 +1258,7 @@
         </is>
       </c>
       <c r="B52" s="5" t="n">
-        <v>1787.95</v>
+        <v>1922.95</v>
       </c>
     </row>
     <row r="53">
@@ -1293,7 +1293,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D46"/>
+  <dimension ref="A1:D47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1787,32 +1787,48 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Uncategorized</t>
+          <t>Leben</t>
         </is>
       </c>
       <c r="B45" s="5" t="n">
-        <v>69.05</v>
+        <v>135</v>
       </c>
       <c r="C45" s="5" t="n">
-        <v>46.2</v>
+        <v>0</v>
       </c>
       <c r="D45" s="5" t="n">
-        <v>22.85</v>
+        <v>135</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
+          <t>Uncategorized</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>69.05</v>
+      </c>
+      <c r="C46" s="5" t="n">
+        <v>46.2</v>
+      </c>
+      <c r="D46" s="5" t="n">
+        <v>22.85</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
           <t>Freizeit</t>
         </is>
       </c>
-      <c r="B46" s="5" t="n">
+      <c r="B47" s="5" t="n">
         <v>100</v>
       </c>
-      <c r="C46" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D46" s="5" t="n">
+      <c r="C47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D47" s="5" t="n">
         <v>100</v>
       </c>
     </row>
@@ -1827,7 +1843,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E54"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2641,21 +2657,63 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
+          <t>Leben</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Gesundheit</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="n">
+        <v>120</v>
+      </c>
+      <c r="D54" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E54" s="5" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Leben</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Familie</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="D55" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E55" s="5" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
           <t>Wohnen</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
+      <c r="B56" t="inlineStr">
         <is>
           <t>Miete und Hypothek</t>
         </is>
       </c>
-      <c r="C54" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D54" s="5" t="n">
+      <c r="C56" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D56" s="5" t="n">
         <v>1774</v>
       </c>
-      <c r="E54" s="5" t="n">
+      <c r="E56" s="5" t="n">
         <v>-1774</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Moves transactions with a Krankenkasse to the separate "Leben/Krankenkasse" subcategory (makes it easier for budgeting).
</commit_message>
<xml_diff>
--- a/data/example/output/dataset.analysis.xlsx
+++ b/data/example/output/dataset.analysis.xlsx
@@ -1843,7 +1843,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E56"/>
+  <dimension ref="A1:E57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2334,17 +2334,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Gesundheit</t>
+          <t>Krankenkasse</t>
         </is>
       </c>
       <c r="C35" s="5" t="n">
         <v>1787.95</v>
       </c>
       <c r="D35" s="5" t="n">
-        <v>101.85</v>
+        <v>77.45</v>
       </c>
       <c r="E35" s="5" t="n">
-        <v>1686.1</v>
+        <v>1710.5</v>
       </c>
     </row>
     <row r="36">
@@ -2413,43 +2413,43 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Mobilität</t>
+          <t>Leben</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Öffentlicher Verkehr</t>
+          <t>Gesundheit</t>
         </is>
       </c>
       <c r="C39" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D39" s="5" t="n">
-        <v>96.90000000000001</v>
+        <v>24.4</v>
       </c>
       <c r="E39" s="5" t="n">
-        <v>-96.90000000000001</v>
+        <v>-24.4</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Wohnen</t>
+          <t>Mobilität</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Miete und Hypothek</t>
+          <t>Öffentlicher Verkehr</t>
         </is>
       </c>
       <c r="C40" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D40" s="5" t="n">
-        <v>1774</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="E40" s="5" t="n">
-        <v>-1774</v>
+        <v>-96.90000000000001</v>
       </c>
     </row>
     <row r="41">
@@ -2460,17 +2460,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Kommunikation</t>
+          <t>Miete und Hypothek</t>
         </is>
       </c>
       <c r="C41" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D41" s="5" t="n">
-        <v>70.27</v>
+        <v>1774</v>
       </c>
       <c r="E41" s="5" t="n">
-        <v>-70.27</v>
+        <v>-1774</v>
       </c>
     </row>
     <row r="42">
@@ -2481,17 +2481,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Haushalt</t>
+          <t>Kommunikation</t>
         </is>
       </c>
       <c r="C42" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D42" s="5" t="n">
-        <v>23.95</v>
+        <v>70.27</v>
       </c>
       <c r="E42" s="5" t="n">
-        <v>-23.95</v>
+        <v>-70.27</v>
       </c>
     </row>
     <row r="43">
@@ -2502,114 +2502,114 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
+          <t>Haushalt</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D43" s="5" t="n">
+        <v>23.95</v>
+      </c>
+      <c r="E43" s="5" t="n">
+        <v>-23.95</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Wohnen</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
           <t>Handwerk und Garten</t>
         </is>
       </c>
-      <c r="C43" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D43" s="5" t="n">
+      <c r="C44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D44" s="5" t="n">
         <v>10.9</v>
       </c>
-      <c r="E43" s="5" t="n">
+      <c r="E44" s="5" t="n">
         <v>-10.9</v>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="3" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
         <is>
           <t>April 2025</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="4" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B48" s="4" t="inlineStr">
+      <c r="B49" s="4" t="inlineStr">
         <is>
           <t>Subcategory</t>
         </is>
       </c>
-      <c r="C48" s="4" t="inlineStr">
+      <c r="C49" s="4" t="inlineStr">
         <is>
           <t>Credit in CHF</t>
         </is>
       </c>
-      <c r="D48" s="4" t="inlineStr">
+      <c r="D49" s="4" t="inlineStr">
         <is>
           <t>Debit in CHF</t>
         </is>
       </c>
-      <c r="E48" s="4" t="inlineStr">
+      <c r="E49" s="4" t="inlineStr">
         <is>
           <t>Net in CHF</t>
         </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>Einkaufen</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>Supermärkte</t>
-        </is>
-      </c>
-      <c r="C49" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D49" s="5" t="n">
-        <v>361.65</v>
-      </c>
-      <c r="E49" s="5" t="n">
-        <v>-361.65</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Einkommen</t>
+          <t>Einkaufen</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Lohn</t>
+          <t>Supermärkte</t>
         </is>
       </c>
       <c r="C50" s="5" t="n">
-        <v>4200</v>
+        <v>0</v>
       </c>
       <c r="D50" s="5" t="n">
-        <v>0</v>
+        <v>361.65</v>
       </c>
       <c r="E50" s="5" t="n">
-        <v>4200</v>
+        <v>-361.65</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Finanzen</t>
+          <t>Einkommen</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Bargeldbezug</t>
+          <t>Lohn</t>
         </is>
       </c>
       <c r="C51" s="5" t="n">
-        <v>0</v>
+        <v>4200</v>
       </c>
       <c r="D51" s="5" t="n">
-        <v>143.5</v>
+        <v>0</v>
       </c>
       <c r="E51" s="5" t="n">
-        <v>-143.5</v>
+        <v>4200</v>
       </c>
     </row>
     <row r="52">
@@ -2620,59 +2620,59 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Spenden</t>
+          <t>Bargeldbezug</t>
         </is>
       </c>
       <c r="C52" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D52" s="5" t="n">
-        <v>25</v>
+        <v>143.5</v>
       </c>
       <c r="E52" s="5" t="n">
-        <v>-25</v>
+        <v>-143.5</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Freizeit</t>
+          <t>Finanzen</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Reisen und Erleben</t>
+          <t>Spenden</t>
         </is>
       </c>
       <c r="C53" s="5" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="D53" s="5" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="E53" s="5" t="n">
-        <v>100</v>
+        <v>-25</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Leben</t>
+          <t>Freizeit</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Gesundheit</t>
+          <t>Reisen und Erleben</t>
         </is>
       </c>
       <c r="C54" s="5" t="n">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="D54" s="5" t="n">
         <v>0</v>
       </c>
       <c r="E54" s="5" t="n">
-        <v>120</v>
+        <v>100</v>
       </c>
     </row>
     <row r="55">
@@ -2683,37 +2683,58 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Familie</t>
+          <t>Krankenkasse</t>
         </is>
       </c>
       <c r="C55" s="5" t="n">
-        <v>15</v>
+        <v>120</v>
       </c>
       <c r="D55" s="5" t="n">
         <v>0</v>
       </c>
       <c r="E55" s="5" t="n">
-        <v>15</v>
+        <v>120</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
+          <t>Leben</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Familie</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="D56" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E56" s="5" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
           <t>Wohnen</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr">
+      <c r="B57" t="inlineStr">
         <is>
           <t>Miete und Hypothek</t>
         </is>
       </c>
-      <c r="C56" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D56" s="5" t="n">
+      <c r="C57" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D57" s="5" t="n">
         <v>1774</v>
       </c>
-      <c r="E56" s="5" t="n">
+      <c r="E57" s="5" t="n">
         <v>-1774</v>
       </c>
     </row>

</xml_diff>